<commit_message>
chained commands added to script indicator
</commit_message>
<xml_diff>
--- a/G7 Commands List.xlsx
+++ b/G7 Commands List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\Serial-Opcode-Sender-LabVIEW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA7E718D-8316-4501-B58D-E1B8B7757867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92E164B-7B1E-4152-81C5-4A020C7809C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="10044" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
   </bookViews>
   <sheets>
     <sheet name="G7 Commands List" sheetId="1" r:id="rId1"/>
@@ -20,147 +20,144 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>command name</t>
   </si>
   <si>
-    <t>header</t>
-  </si>
-  <si>
-    <t>length</t>
-  </si>
-  <si>
-    <t>cmd opcode</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>checksum</t>
-  </si>
-  <si>
     <t>response length (bytes)</t>
   </si>
   <si>
-    <t>SET DUT to advertise &amp; wakeup DUT</t>
-  </si>
-  <si>
-    <t>0xAA</t>
-  </si>
-  <si>
-    <t>0x08</t>
-  </si>
-  <si>
-    <t>0x4B</t>
-  </si>
-  <si>
-    <t>0x01 0x01 0x00 0x00 0xD0 0x07</t>
-  </si>
-  <si>
-    <t>0x94</t>
-  </si>
-  <si>
-    <t>GET TXSN &amp; FW version</t>
-  </si>
-  <si>
-    <t>0x02</t>
-  </si>
-  <si>
-    <t>0x4A</t>
-  </si>
-  <si>
-    <t>0x48</t>
-  </si>
-  <si>
-    <t>GET DUT temp</t>
-  </si>
-  <si>
-    <t>0xC2</t>
-  </si>
-  <si>
-    <t>0xC0</t>
-  </si>
-  <si>
-    <t>GET battery voltages</t>
-  </si>
-  <si>
-    <t>0x22</t>
-  </si>
-  <si>
-    <t>0x20</t>
-  </si>
-  <si>
-    <t>SET battery type</t>
-  </si>
-  <si>
-    <t>0x04</t>
-  </si>
-  <si>
-    <t>0x56</t>
-  </si>
-  <si>
-    <t>0x00 0x05</t>
-  </si>
-  <si>
-    <t>0x57</t>
-  </si>
-  <si>
-    <t>SET TOM1</t>
-  </si>
-  <si>
-    <t>0x07</t>
-  </si>
-  <si>
-    <t>0x95</t>
-  </si>
-  <si>
-    <t>0x01 0x63 0x4F 0x77 0x35</t>
-  </si>
-  <si>
-    <t>0xFD</t>
-  </si>
-  <si>
-    <t>Commit TOM1 &amp; battery type to NVM followed by soft-reset</t>
-  </si>
-  <si>
-    <t>0x03</t>
-  </si>
-  <si>
-    <t>0x31</t>
-  </si>
-  <si>
-    <t>0x00</t>
-  </si>
-  <si>
-    <t>0x32</t>
-  </si>
-  <si>
-    <t>GET battery type</t>
-  </si>
-  <si>
-    <t>0x55</t>
-  </si>
-  <si>
-    <t>GET TOM1</t>
-  </si>
-  <si>
-    <t>0x97</t>
-  </si>
-  <si>
-    <t>Disable UART</t>
-  </si>
-  <si>
-    <t>0x7C</t>
-  </si>
-  <si>
-    <t>0x7B</t>
-  </si>
-  <si>
-    <t>SET storage mode (mode 2)</t>
-  </si>
-  <si>
-    <t>0x7D</t>
+    <t>0x31: Reset</t>
+  </si>
+  <si>
+    <t>0xB3: Set RTS 0</t>
+  </si>
+  <si>
+    <t>0xB3: Get RTS</t>
+  </si>
+  <si>
+    <t>0x4A: GET TXSN &amp; FW</t>
+  </si>
+  <si>
+    <t>0x92: Get Pairing Code</t>
+  </si>
+  <si>
+    <t>0x91: Get TXSN</t>
+  </si>
+  <si>
+    <t>0x22: Get Battery Voltages</t>
+  </si>
+  <si>
+    <t>0x74: Get TMR Battery Presence</t>
+  </si>
+  <si>
+    <t>0x93: Get State (FTM Get State)</t>
+  </si>
+  <si>
+    <t>0x97: Get TOMs</t>
+  </si>
+  <si>
+    <t>0x95: SET TOM1</t>
+  </si>
+  <si>
+    <t>0x56: Set Battery (2) Maxell</t>
+  </si>
+  <si>
+    <t>0x56: Set Battery (6) Murata</t>
+  </si>
+  <si>
+    <t>0x56: Set Battery (5) Panasonic</t>
+  </si>
+  <si>
+    <t>0x56: GET battery type</t>
+  </si>
+  <si>
+    <t>0xC2: Get Temperature</t>
+  </si>
+  <si>
+    <t>0x4D: Set FTM (CGM to FTM)</t>
+  </si>
+  <si>
+    <t>0x6E: Set (Toggle) BLE ON</t>
+  </si>
+  <si>
+    <t>0x6E: Set (Toggle) BLE OFF</t>
+  </si>
+  <si>
+    <t>0x7A: Get M0&amp;Mf</t>
+  </si>
+  <si>
+    <t>0x7A: SET M0&amp;Mf to default</t>
+  </si>
+  <si>
+    <t>0x64: SET SIV Parameters</t>
+  </si>
+  <si>
+    <t>0x7E: Check Sensor</t>
+  </si>
+  <si>
+    <t>0x7C (5): SET FTM Complete</t>
+  </si>
+  <si>
+    <t>0x7C (2): SET Storage Mode</t>
+  </si>
+  <si>
+    <t>0x7C (4): SET Disable_UART</t>
+  </si>
+  <si>
+    <t>0x7C (8): SET Unrestrict_NFC</t>
+  </si>
+  <si>
+    <t>0x7C (9): SET Disable_Security</t>
+  </si>
+  <si>
+    <t>0x7C (10): SET Enable_UART</t>
+  </si>
+  <si>
+    <t>0x4B: SET DUT to advertise &amp; wakeup DUT</t>
+  </si>
+  <si>
+    <t>Command</t>
+  </si>
+  <si>
+    <t>0xAA 0x08 0x4B 0x01 0x01 0x00 0x00 0xD0 0x07 0x94</t>
+  </si>
+  <si>
+    <t>0xAA 0x03 0x32 0x00 0x32</t>
+  </si>
+  <si>
+    <t>0xAA 0x02 0x4A 0x48</t>
+  </si>
+  <si>
+    <t>0xAA 0x02 0x22 0x20</t>
+  </si>
+  <si>
+    <t>0xAA 0x02 0x97 0x95</t>
+  </si>
+  <si>
+    <t>0xAA 0x07 0x95 0x01 0x63 0x4F 0x77 0x35 0xFD</t>
+  </si>
+  <si>
+    <t>0xAA 0xx04 0x56 0x00 0x02 ?</t>
+  </si>
+  <si>
+    <t>0xAA 0xx04 0x56 0x00 0x06 ?</t>
+  </si>
+  <si>
+    <t>0xAA 0xx04 0x56 0x00 0x05 57</t>
+  </si>
+  <si>
+    <t>0xAA 0x03 0x56 0x00 0x55</t>
+  </si>
+  <si>
+    <t>0xAA 0x02 0xC2 0xC0</t>
+  </si>
+  <si>
+    <t>0xAA 0x03 0x7C 0x02 0x7D</t>
+  </si>
+  <si>
+    <t>0xAA 0x03 0x7C 0x04 0x7B</t>
   </si>
 </sst>
 </file>
@@ -1021,271 +1018,251 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A1A2F9-EB88-4036-A12E-635F91F6E518}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="57.88671875" customWidth="1"/>
+    <col min="2" max="2" width="54.109375" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="G2">
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B28" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>28</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>29</v>
       </c>
-      <c r="D7" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>30</v>
-      </c>
-      <c r="E7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G9">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G12">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
send single and chained cmds implemented
</commit_message>
<xml_diff>
--- a/G7 Commands List.xlsx
+++ b/G7 Commands List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\Serial-Opcode-Sender-LabVIEW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92E164B-7B1E-4152-81C5-4A020C7809C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A2AA5F-156C-4F21-AFF6-36D3BD50F2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
+    <workbookView xWindow="2952" yWindow="912" windowWidth="17280" windowHeight="10044" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
   </bookViews>
   <sheets>
     <sheet name="G7 Commands List" sheetId="1" r:id="rId1"/>
@@ -28,136 +28,136 @@
     <t>response length (bytes)</t>
   </si>
   <si>
-    <t>0x31: Reset</t>
-  </si>
-  <si>
-    <t>0xB3: Set RTS 0</t>
-  </si>
-  <si>
-    <t>0xB3: Get RTS</t>
-  </si>
-  <si>
-    <t>0x4A: GET TXSN &amp; FW</t>
-  </si>
-  <si>
-    <t>0x92: Get Pairing Code</t>
-  </si>
-  <si>
-    <t>0x91: Get TXSN</t>
-  </si>
-  <si>
-    <t>0x22: Get Battery Voltages</t>
-  </si>
-  <si>
-    <t>0x74: Get TMR Battery Presence</t>
-  </si>
-  <si>
-    <t>0x93: Get State (FTM Get State)</t>
-  </si>
-  <si>
-    <t>0x97: Get TOMs</t>
-  </si>
-  <si>
-    <t>0x95: SET TOM1</t>
-  </si>
-  <si>
-    <t>0x56: Set Battery (2) Maxell</t>
-  </si>
-  <si>
-    <t>0x56: Set Battery (6) Murata</t>
-  </si>
-  <si>
-    <t>0x56: Set Battery (5) Panasonic</t>
-  </si>
-  <si>
-    <t>0x56: GET battery type</t>
-  </si>
-  <si>
-    <t>0xC2: Get Temperature</t>
-  </si>
-  <si>
-    <t>0x4D: Set FTM (CGM to FTM)</t>
-  </si>
-  <si>
-    <t>0x6E: Set (Toggle) BLE ON</t>
-  </si>
-  <si>
-    <t>0x6E: Set (Toggle) BLE OFF</t>
-  </si>
-  <si>
-    <t>0x7A: Get M0&amp;Mf</t>
-  </si>
-  <si>
-    <t>0x7A: SET M0&amp;Mf to default</t>
-  </si>
-  <si>
-    <t>0x64: SET SIV Parameters</t>
-  </si>
-  <si>
-    <t>0x7E: Check Sensor</t>
-  </si>
-  <si>
-    <t>0x7C (5): SET FTM Complete</t>
-  </si>
-  <si>
-    <t>0x7C (2): SET Storage Mode</t>
-  </si>
-  <si>
-    <t>0x7C (4): SET Disable_UART</t>
-  </si>
-  <si>
-    <t>0x7C (8): SET Unrestrict_NFC</t>
-  </si>
-  <si>
-    <t>0x7C (9): SET Disable_Security</t>
-  </si>
-  <si>
-    <t>0x7C (10): SET Enable_UART</t>
-  </si>
-  <si>
-    <t>0x4B: SET DUT to advertise &amp; wakeup DUT</t>
-  </si>
-  <si>
     <t>Command</t>
   </si>
   <si>
-    <t>0xAA 0x08 0x4B 0x01 0x01 0x00 0x00 0xD0 0x07 0x94</t>
-  </si>
-  <si>
-    <t>0xAA 0x03 0x32 0x00 0x32</t>
-  </si>
-  <si>
-    <t>0xAA 0x02 0x4A 0x48</t>
-  </si>
-  <si>
-    <t>0xAA 0x02 0x22 0x20</t>
-  </si>
-  <si>
-    <t>0xAA 0x02 0x97 0x95</t>
-  </si>
-  <si>
-    <t>0xAA 0x07 0x95 0x01 0x63 0x4F 0x77 0x35 0xFD</t>
-  </si>
-  <si>
-    <t>0xAA 0xx04 0x56 0x00 0x02 ?</t>
-  </si>
-  <si>
-    <t>0xAA 0xx04 0x56 0x00 0x06 ?</t>
-  </si>
-  <si>
-    <t>0xAA 0xx04 0x56 0x00 0x05 57</t>
-  </si>
-  <si>
-    <t>0xAA 0x03 0x56 0x00 0x55</t>
-  </si>
-  <si>
-    <t>0xAA 0x02 0xC2 0xC0</t>
-  </si>
-  <si>
-    <t>0xAA 0x03 0x7C 0x02 0x7D</t>
-  </si>
-  <si>
-    <t>0xAA 0x03 0x7C 0x04 0x7B</t>
+    <t>4B: SET DUT to advertise &amp; wakeup DUT</t>
+  </si>
+  <si>
+    <t>AA 08 4B 01 01 00 00 D0 07 94</t>
+  </si>
+  <si>
+    <t>31: Reset</t>
+  </si>
+  <si>
+    <t>AA 03 32 00 32</t>
+  </si>
+  <si>
+    <t>B3: Set RTS 0</t>
+  </si>
+  <si>
+    <t>B3: Get RTS</t>
+  </si>
+  <si>
+    <t>4A: GET TXSN &amp; FW</t>
+  </si>
+  <si>
+    <t>92: Get Pairing Code</t>
+  </si>
+  <si>
+    <t>91: Get TXSN</t>
+  </si>
+  <si>
+    <t>22: Get Battery Voltages</t>
+  </si>
+  <si>
+    <t>AA 02 22 20</t>
+  </si>
+  <si>
+    <t>74: Get TMR Battery Presence</t>
+  </si>
+  <si>
+    <t>93: Get State (FTM Get State)</t>
+  </si>
+  <si>
+    <t>97: Get TOMs</t>
+  </si>
+  <si>
+    <t>AA 02 97 95</t>
+  </si>
+  <si>
+    <t>95: SET TOM1</t>
+  </si>
+  <si>
+    <t>AA 07 95 01 63 4F 77 35 FD</t>
+  </si>
+  <si>
+    <t>56: Set Battery (2) Maxell</t>
+  </si>
+  <si>
+    <t>AA x04 56 00 02 ?</t>
+  </si>
+  <si>
+    <t>56: Set Battery (6) Murata</t>
+  </si>
+  <si>
+    <t>AA x04 56 00 06 ?</t>
+  </si>
+  <si>
+    <t>56: Set Battery (5) Panasonic</t>
+  </si>
+  <si>
+    <t>AA x04 56 00 05 57</t>
+  </si>
+  <si>
+    <t>56: GET battery type</t>
+  </si>
+  <si>
+    <t>AA 03 56 00 55</t>
+  </si>
+  <si>
+    <t>C2: Get Temperature</t>
+  </si>
+  <si>
+    <t>AA 02 C2 C0</t>
+  </si>
+  <si>
+    <t>4D: Set FTM (CGM to FTM)</t>
+  </si>
+  <si>
+    <t>6E: Set (Toggle) BLE ON</t>
+  </si>
+  <si>
+    <t>6E: Set (Toggle) BLE OFF</t>
+  </si>
+  <si>
+    <t>7A: Get M0&amp;Mf</t>
+  </si>
+  <si>
+    <t>7A: SET M0&amp;Mf to default</t>
+  </si>
+  <si>
+    <t>64: SET SIV Parameters</t>
+  </si>
+  <si>
+    <t>7E: Check Sensor</t>
+  </si>
+  <si>
+    <t>7C (5): SET FTM Complete</t>
+  </si>
+  <si>
+    <t>7C (2): SET Storage Mode</t>
+  </si>
+  <si>
+    <t>AA 03 7C 02 7D</t>
+  </si>
+  <si>
+    <t>7C (4): SET Disable_UART</t>
+  </si>
+  <si>
+    <t>AA 03 7C 04 7B</t>
+  </si>
+  <si>
+    <t>7C (8): SET Unrestrict_NFC</t>
+  </si>
+  <si>
+    <t>7C (9): SET Disable_Security</t>
+  </si>
+  <si>
+    <t>7C (10): SET Enable_UART</t>
+  </si>
+  <si>
+    <t>AA 02 4A 48</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1031,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1039,10 +1039,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>15</v>
@@ -1050,10 +1050,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>5</v>
@@ -1061,20 +1061,20 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C6">
         <v>27</v>
@@ -1082,20 +1082,20 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -1103,20 +1103,20 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="C12">
         <v>21</v>
@@ -1124,10 +1124,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C13">
         <v>18</v>
@@ -1135,10 +1135,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="C14">
         <v>14</v>
@@ -1146,10 +1146,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -1157,10 +1157,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C16">
         <v>14</v>
@@ -1168,10 +1168,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="C17">
         <v>13</v>
@@ -1179,10 +1179,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="C18">
         <v>14</v>
@@ -1190,50 +1190,50 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C27">
         <v>12</v>
@@ -1241,10 +1241,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C28">
         <v>12</v>
@@ -1252,17 +1252,17 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated com port error handling
</commit_message>
<xml_diff>
--- a/G7 Commands List.xlsx
+++ b/G7 Commands List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\Serial-Opcode-Sender-LabVIEW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A2AA5F-156C-4F21-AFF6-36D3BD50F2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC1714F-7CBF-48CD-BD63-B8C0D2177C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2952" yWindow="912" windowWidth="17280" windowHeight="10044" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
+    <workbookView xWindow="1236" yWindow="1116" windowWidth="17280" windowHeight="12300" xr2:uid="{4B944086-30BA-48E8-9A36-5C26F7877D52}"/>
   </bookViews>
   <sheets>
     <sheet name="G7 Commands List" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>command name</t>
   </si>
@@ -28,9 +28,6 @@
     <t>response length (bytes)</t>
   </si>
   <si>
-    <t>Command</t>
-  </si>
-  <si>
     <t>4B: SET DUT to advertise &amp; wakeup DUT</t>
   </si>
   <si>
@@ -85,21 +82,12 @@
     <t>56: Set Battery (2) Maxell</t>
   </si>
   <si>
-    <t>AA x04 56 00 02 ?</t>
-  </si>
-  <si>
     <t>56: Set Battery (6) Murata</t>
   </si>
   <si>
-    <t>AA x04 56 00 06 ?</t>
-  </si>
-  <si>
     <t>56: Set Battery (5) Panasonic</t>
   </si>
   <si>
-    <t>AA x04 56 00 05 57</t>
-  </si>
-  <si>
     <t>56: GET battery type</t>
   </si>
   <si>
@@ -115,12 +103,6 @@
     <t>4D: Set FTM (CGM to FTM)</t>
   </si>
   <si>
-    <t>6E: Set (Toggle) BLE ON</t>
-  </si>
-  <si>
-    <t>6E: Set (Toggle) BLE OFF</t>
-  </si>
-  <si>
     <t>7A: Get M0&amp;Mf</t>
   </si>
   <si>
@@ -158,6 +140,69 @@
   </si>
   <si>
     <t>AA 02 4A 48</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Not variable</t>
+  </si>
+  <si>
+    <t>AA 02 91 93</t>
+  </si>
+  <si>
+    <t>command</t>
+  </si>
+  <si>
+    <t>AA 02 4D 4F</t>
+  </si>
+  <si>
+    <t>AA 03 7C 05 ?</t>
+  </si>
+  <si>
+    <t>AA 03 74 00 77</t>
+  </si>
+  <si>
+    <t>AA 02 93 91</t>
+  </si>
+  <si>
+    <t>AA 03 7C 08 ?</t>
+  </si>
+  <si>
+    <t>AA 03 7C 09 ?</t>
+  </si>
+  <si>
+    <t>AA 03 7C 10 ?</t>
+  </si>
+  <si>
+    <t>need to look into command more / get checksum</t>
+  </si>
+  <si>
+    <t>AA 02 B3 B1</t>
+  </si>
+  <si>
+    <t>AA 04 B3 01 00 B6</t>
+  </si>
+  <si>
+    <t>AA 02 92 90</t>
+  </si>
+  <si>
+    <t>AA 04 56 00 02 50</t>
+  </si>
+  <si>
+    <t>AA 04 56 00 06 54</t>
+  </si>
+  <si>
+    <t>AA 04 56 00 05 57</t>
+  </si>
+  <si>
+    <t>AA 02 7A 78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AA 12 7A 00 00 C0 41 00 00 F0 41 00 00 88 41 00 00 90 41 40 </t>
+  </si>
+  <si>
+    <t>AA 09 7E 01 00 00 E8 03 00 00 9D</t>
   </si>
 </sst>
 </file>
@@ -300,7 +345,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -478,6 +523,24 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -641,8 +704,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1018,251 +1084,328 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A1A2F9-EB88-4036-A12E-635F91F6E518}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="57.88671875" customWidth="1"/>
     <col min="2" max="2" width="54.109375" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="3">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3">
+        <v>5</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="3">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="3"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="C6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="C24" s="3">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="B25" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="C25" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="B26" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="C26" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="B27" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B27" t="s">
-        <v>39</v>
-      </c>
-      <c r="C27">
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="3">
         <v>12</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>